<commit_message>
feat: correções paper e code
</commit_message>
<xml_diff>
--- a/batch_pre_sizing_casos_materia.xlsx
+++ b/batch_pre_sizing_casos_materia.xlsx
@@ -727,22 +727,22 @@
         <v>20</v>
       </c>
       <c r="Z2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA2" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB2" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD2" t="n">
         <v>5</v>
       </c>
       <c r="AE2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF2" t="n">
         <v>30</v>
@@ -760,7 +760,7 @@
         <v>50</v>
       </c>
       <c r="AK2" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL2" t="n">
         <v>30</v>
@@ -774,7 +774,6 @@
       <c r="AO2" t="b">
         <v>1</v>
       </c>
-      <c r="AP2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -863,22 +862,22 @@
         <v>30</v>
       </c>
       <c r="Z3" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA3" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB3" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD3" t="n">
         <v>5</v>
       </c>
       <c r="AE3" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF3" t="n">
         <v>30</v>
@@ -896,7 +895,7 @@
         <v>50</v>
       </c>
       <c r="AK3" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL3" t="n">
         <v>30</v>
@@ -910,7 +909,6 @@
       <c r="AO3" t="b">
         <v>1</v>
       </c>
-      <c r="AP3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -999,22 +997,22 @@
         <v>40</v>
       </c>
       <c r="Z4" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA4" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC4" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD4" t="n">
         <v>5</v>
       </c>
       <c r="AE4" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF4" t="n">
         <v>30</v>
@@ -1032,7 +1030,7 @@
         <v>50</v>
       </c>
       <c r="AK4" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL4" t="n">
         <v>30</v>
@@ -1046,7 +1044,6 @@
       <c r="AO4" t="b">
         <v>1</v>
       </c>
-      <c r="AP4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1135,22 +1132,22 @@
         <v>50</v>
       </c>
       <c r="Z5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB5" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC5" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD5" t="n">
         <v>5</v>
       </c>
       <c r="AE5" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF5" t="n">
         <v>30</v>
@@ -1168,7 +1165,7 @@
         <v>50</v>
       </c>
       <c r="AK5" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL5" t="n">
         <v>30</v>
@@ -1182,7 +1179,6 @@
       <c r="AO5" t="b">
         <v>1</v>
       </c>
-      <c r="AP5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1271,22 +1267,22 @@
         <v>60</v>
       </c>
       <c r="Z6" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA6" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB6" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC6" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD6" t="n">
         <v>5</v>
       </c>
       <c r="AE6" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF6" t="n">
         <v>30</v>
@@ -1304,7 +1300,7 @@
         <v>50</v>
       </c>
       <c r="AK6" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL6" t="n">
         <v>30</v>
@@ -1318,7 +1314,6 @@
       <c r="AO6" t="b">
         <v>1</v>
       </c>
-      <c r="AP6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1407,22 +1402,22 @@
         <v>20</v>
       </c>
       <c r="Z7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA7" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB7" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD7" t="n">
         <v>5</v>
       </c>
       <c r="AE7" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF7" t="n">
         <v>30</v>
@@ -1440,7 +1435,7 @@
         <v>50</v>
       </c>
       <c r="AK7" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL7" t="n">
         <v>30</v>
@@ -1454,7 +1449,6 @@
       <c r="AO7" t="b">
         <v>1</v>
       </c>
-      <c r="AP7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1543,22 +1537,22 @@
         <v>30</v>
       </c>
       <c r="Z8" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA8" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB8" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD8" t="n">
         <v>5</v>
       </c>
       <c r="AE8" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF8" t="n">
         <v>30</v>
@@ -1576,7 +1570,7 @@
         <v>50</v>
       </c>
       <c r="AK8" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL8" t="n">
         <v>30</v>
@@ -1590,7 +1584,6 @@
       <c r="AO8" t="b">
         <v>1</v>
       </c>
-      <c r="AP8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1679,22 +1672,22 @@
         <v>40</v>
       </c>
       <c r="Z9" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA9" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB9" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD9" t="n">
         <v>5</v>
       </c>
       <c r="AE9" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF9" t="n">
         <v>30</v>
@@ -1712,7 +1705,7 @@
         <v>50</v>
       </c>
       <c r="AK9" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL9" t="n">
         <v>30</v>
@@ -1726,7 +1719,6 @@
       <c r="AO9" t="b">
         <v>1</v>
       </c>
-      <c r="AP9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1815,22 +1807,22 @@
         <v>50</v>
       </c>
       <c r="Z10" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA10" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB10" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC10" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD10" t="n">
         <v>5</v>
       </c>
       <c r="AE10" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF10" t="n">
         <v>30</v>
@@ -1848,7 +1840,7 @@
         <v>50</v>
       </c>
       <c r="AK10" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL10" t="n">
         <v>30</v>
@@ -1862,7 +1854,6 @@
       <c r="AO10" t="b">
         <v>1</v>
       </c>
-      <c r="AP10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1951,22 +1942,22 @@
         <v>60</v>
       </c>
       <c r="Z11" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA11" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB11" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC11" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD11" t="n">
         <v>5</v>
       </c>
       <c r="AE11" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF11" t="n">
         <v>30</v>
@@ -1984,7 +1975,7 @@
         <v>50</v>
       </c>
       <c r="AK11" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL11" t="n">
         <v>30</v>
@@ -1998,7 +1989,6 @@
       <c r="AO11" t="b">
         <v>1</v>
       </c>
-      <c r="AP11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2087,22 +2077,22 @@
         <v>20</v>
       </c>
       <c r="Z12" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA12" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB12" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC12" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD12" t="n">
         <v>5</v>
       </c>
       <c r="AE12" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF12" t="n">
         <v>30</v>
@@ -2120,7 +2110,7 @@
         <v>50</v>
       </c>
       <c r="AK12" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL12" t="n">
         <v>30</v>
@@ -2134,7 +2124,6 @@
       <c r="AO12" t="b">
         <v>1</v>
       </c>
-      <c r="AP12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2223,22 +2212,22 @@
         <v>30</v>
       </c>
       <c r="Z13" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA13" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB13" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC13" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD13" t="n">
         <v>5</v>
       </c>
       <c r="AE13" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF13" t="n">
         <v>30</v>
@@ -2256,7 +2245,7 @@
         <v>50</v>
       </c>
       <c r="AK13" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL13" t="n">
         <v>30</v>
@@ -2270,7 +2259,6 @@
       <c r="AO13" t="b">
         <v>1</v>
       </c>
-      <c r="AP13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2359,22 +2347,22 @@
         <v>40</v>
       </c>
       <c r="Z14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA14" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB14" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC14" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD14" t="n">
         <v>5</v>
       </c>
       <c r="AE14" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF14" t="n">
         <v>30</v>
@@ -2392,7 +2380,7 @@
         <v>50</v>
       </c>
       <c r="AK14" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL14" t="n">
         <v>30</v>
@@ -2406,7 +2394,6 @@
       <c r="AO14" t="b">
         <v>1</v>
       </c>
-      <c r="AP14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2495,22 +2482,22 @@
         <v>50</v>
       </c>
       <c r="Z15" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA15" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB15" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC15" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD15" t="n">
         <v>5</v>
       </c>
       <c r="AE15" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF15" t="n">
         <v>30</v>
@@ -2528,7 +2515,7 @@
         <v>50</v>
       </c>
       <c r="AK15" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL15" t="n">
         <v>30</v>
@@ -2542,7 +2529,6 @@
       <c r="AO15" t="b">
         <v>1</v>
       </c>
-      <c r="AP15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2631,22 +2617,22 @@
         <v>60</v>
       </c>
       <c r="Z16" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA16" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB16" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC16" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD16" t="n">
         <v>5</v>
       </c>
       <c r="AE16" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF16" t="n">
         <v>30</v>
@@ -2664,7 +2650,7 @@
         <v>50</v>
       </c>
       <c r="AK16" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL16" t="n">
         <v>30</v>
@@ -2678,7 +2664,6 @@
       <c r="AO16" t="b">
         <v>1</v>
       </c>
-      <c r="AP16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2767,22 +2752,22 @@
         <v>20</v>
       </c>
       <c r="Z17" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA17" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB17" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC17" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD17" t="n">
         <v>5</v>
       </c>
       <c r="AE17" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF17" t="n">
         <v>30</v>
@@ -2800,7 +2785,7 @@
         <v>50</v>
       </c>
       <c r="AK17" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL17" t="n">
         <v>30</v>
@@ -2814,7 +2799,6 @@
       <c r="AO17" t="b">
         <v>1</v>
       </c>
-      <c r="AP17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2903,22 +2887,22 @@
         <v>30</v>
       </c>
       <c r="Z18" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA18" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB18" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC18" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD18" t="n">
         <v>5</v>
       </c>
       <c r="AE18" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF18" t="n">
         <v>30</v>
@@ -2936,7 +2920,7 @@
         <v>50</v>
       </c>
       <c r="AK18" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL18" t="n">
         <v>30</v>
@@ -2950,7 +2934,6 @@
       <c r="AO18" t="b">
         <v>1</v>
       </c>
-      <c r="AP18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3039,22 +3022,22 @@
         <v>40</v>
       </c>
       <c r="Z19" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA19" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB19" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC19" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD19" t="n">
         <v>5</v>
       </c>
       <c r="AE19" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF19" t="n">
         <v>30</v>
@@ -3072,7 +3055,7 @@
         <v>50</v>
       </c>
       <c r="AK19" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL19" t="n">
         <v>30</v>
@@ -3086,7 +3069,6 @@
       <c r="AO19" t="b">
         <v>1</v>
       </c>
-      <c r="AP19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3175,22 +3157,22 @@
         <v>50</v>
       </c>
       <c r="Z20" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA20" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB20" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC20" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD20" t="n">
         <v>5</v>
       </c>
       <c r="AE20" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF20" t="n">
         <v>30</v>
@@ -3208,7 +3190,7 @@
         <v>50</v>
       </c>
       <c r="AK20" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL20" t="n">
         <v>30</v>
@@ -3222,7 +3204,6 @@
       <c r="AO20" t="b">
         <v>1</v>
       </c>
-      <c r="AP20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3311,22 +3292,22 @@
         <v>60</v>
       </c>
       <c r="Z21" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AA21" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="AB21" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AC21" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="AD21" t="n">
         <v>5</v>
       </c>
       <c r="AE21" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AF21" t="n">
         <v>30</v>
@@ -3344,7 +3325,7 @@
         <v>50</v>
       </c>
       <c r="AK21" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="AL21" t="n">
         <v>30</v>
@@ -3358,7 +3339,6 @@
       <c r="AO21" t="b">
         <v>1</v>
       </c>
-      <c r="AP21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>